<commit_message>
Refine RINVOQ homepage to match live site
- Per-brand styles.css folder structure (linzess/, rinvoq/) to isolate
  brand CSS; remove old flat brand sheets
- Hero carousel (2 slides) with object-position 54% 50% crop match
- Savings/About full-bleed split, SPEAK band brushstroke alignment,
  "You could pay" heading, condition cards
- Self-hosted RINVOQ hero images, brushstroke, SPEAK bg + icon SVGs
- RINVOQ importer bundles + pixel-compare tooling
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="203">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,28 +37,589 @@
     <t>url</t>
   </si>
   <si>
+    <t>espanol.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>espanol</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>patient-transcript</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:10:23.135Z</t>
+  </si>
+  <si>
+    <t>El tratamiento de marca más recetado para IBS-C y CIC | LINZESS (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/espanol</t>
+  </si>
+  <si>
+    <t>find-relief.report.json</t>
+  </si>
+  <si>
+    <t>["hero-pharma","tabs-navigation","video-single","video-single","columns-promo","columns-cta"]</t>
+  </si>
+  <si>
+    <t>find-relief</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-06-12T18:00:47.768Z</t>
+  </si>
+  <si>
+    <t>Find Relief | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/find-relief</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-pharma","columns-promo","columns-promo","columns-promo","cards-feature","cards-stats","cards-video"]</t>
+    <t>["hero-pharma","promo-tout","promo-tout","promo-tout","cards-feature","cards-stats","cards-video"]</t>
   </si>
   <si>
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-06-05T18:23:17.030Z</t>
+    <t>2026-06-13T08:03:21.258Z</t>
   </si>
   <si>
     <t>LINZESS (linaclotide) for IBS-C &amp; CIC | Patient Information</t>
   </si>
   <si>
     <t>https://www.linzess.com/</t>
+  </si>
+  <si>
+    <t>page-not-found.report.json</t>
+  </si>
+  <si>
+    <t>page-not-found</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:59.855Z</t>
+  </si>
+  <si>
+    <t>Page Not Found | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/page-not-found</t>
+  </si>
+  <si>
+    <t>resources.report.json</t>
+  </si>
+  <si>
+    <t>["hero-pharma","tabs-navigation","columns-promo","columns-cta"]</t>
+  </si>
+  <si>
+    <t>resources</t>
+  </si>
+  <si>
+    <t>2026-06-08T18:45:29.195Z</t>
+  </si>
+  <si>
+    <t>Resources &amp; Helpful Information | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/resources</t>
+  </si>
+  <si>
+    <t>savings-and-support.report.json</t>
+  </si>
+  <si>
+    <t>savings-and-support</t>
+  </si>
+  <si>
+    <t>2026-06-08T18:45:36.030Z</t>
+  </si>
+  <si>
+    <t>Cost Savings &amp; Financial Support | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/savings-and-support</t>
+  </si>
+  <si>
+    <t>savings-card.report.json</t>
+  </si>
+  <si>
+    <t>savings-card</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:58.641Z</t>
+  </si>
+  <si>
+    <t>Savings Card | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/savings-card</t>
+  </si>
+  <si>
+    <t>search-results.report.json</t>
+  </si>
+  <si>
+    <t>search-results</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:10:08.671Z</t>
+  </si>
+  <si>
+    <t>Search Request | LINZESS (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/search-results</t>
+  </si>
+  <si>
+    <t>sitemap.report.json</t>
+  </si>
+  <si>
+    <t>sitemap</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:52.774Z</t>
+  </si>
+  <si>
+    <t>Sitemap | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/sitemap</t>
+  </si>
+  <si>
+    <t>understanding-constipation.report.json</t>
+  </si>
+  <si>
+    <t>understanding-constipation</t>
+  </si>
+  <si>
+    <t>2026-06-08T18:45:14.957Z</t>
+  </si>
+  <si>
+    <t>Understanding Symptoms &amp; Types of Constipation | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/understanding-constipation</t>
+  </si>
+  <si>
+    <t>why-linzess.report.json</t>
+  </si>
+  <si>
+    <t>["hero-pharma","tabs-navigation","cards-checklist","cards-checklist","cards-icon","cards-icon","cards-video","video-playlist","video-playlist","columns-promo","columns-cta"]</t>
+  </si>
+  <si>
+    <t>why-linzess</t>
+  </si>
+  <si>
+    <t>2026-06-12T18:00:54.771Z</t>
+  </si>
+  <si>
+    <t>What is LINZESS &amp; How Does It Work | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess</t>
+  </si>
+  <si>
+    <t>find-relief/gutcheck.report.json</t>
+  </si>
+  <si>
+    <t>find-relief/gutcheck</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:18.464Z</t>
+  </si>
+  <si>
+    <t>Gut Check Quiz for IBS-C &amp; CIC | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/find-relief/gutcheck</t>
+  </si>
+  <si>
+    <t>find-relief/talk-to-a-doctor.report.json</t>
+  </si>
+  <si>
+    <t>find-relief/talk-to-a-doctor</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:44.186Z</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/find-relief/talk-to-a-doctor</t>
+  </si>
+  <si>
+    <t>savings-and-support/faqs.report.json</t>
+  </si>
+  <si>
+    <t>savings-and-support/faqs</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:25.599Z</t>
+  </si>
+  <si>
+    <t>Frequently Asked Questions | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/savings-and-support/faqs</t>
+  </si>
+  <si>
+    <t>savings-and-support/from-the-gut.report.json</t>
+  </si>
+  <si>
+    <t>savings-and-support/from-the-gut</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:34.876Z</t>
+  </si>
+  <si>
+    <t>Healthy Gut Tips, Recipes &amp; More | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/savings-and-support/from-the-gut</t>
+  </si>
+  <si>
+    <t>savings-card/savings.report.json</t>
+  </si>
+  <si>
+    <t>savings-card/savings</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:09.073Z</t>
+  </si>
+  <si>
+    <t>ERROR: The request could not be satisfied</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/savings-card/savings</t>
+  </si>
+  <si>
+    <t>savings-card/terms.report.json</t>
+  </si>
+  <si>
+    <t>savings-card/terms</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:09:03.386Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://www.linzess.com/savings-card/terms</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:50.901Z</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/healthy-routines</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:42.856Z</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/wellness-tips</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:07:34.353Z</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines/keeping-in-touch-with-your-doctor.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines/keeping-in-touch-with-your-doctor</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:35.155Z</t>
+  </si>
+  <si>
+    <t>Keeping in Touch with Your Doctor | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/healthy-routines/keeping-in-touch-with-your-doctor</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines/otc-and-prescription-treatments.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines/otc-and-prescription-treatments</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:20.338Z</t>
+  </si>
+  <si>
+    <t>OTC and Prescription Treatments | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/healthy-routines/otc-and-prescription-treatments</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines/tackling-ibs-c-triggers.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/healthy-routines/tackling-ibs-c-triggers</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:27.275Z</t>
+  </si>
+  <si>
+    <t>Tackling IBS-C Triggers and Flare-Ups | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/healthy-routines/tackling-ibs-c-triggers</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/5-holiday-low-fodmap-recipes.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/5-holiday-low-fodmap-recipes</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:03.659Z</t>
+  </si>
+  <si>
+    <t>5 Low FODMAP Holiday Recipes | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/wellness-tips/5-holiday-low-fodmap-recipes</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/good-for-your-gut-flavorful-food-swaps.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/good-for-your-gut-flavorful-food-swaps</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:07:48.970Z</t>
+  </si>
+  <si>
+    <t>Helpful Foods for Constipation | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/wellness-tips/good-for-your-gut-flavorful-food-swaps</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/is-your-pantry-fodmap-friendly.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/is-your-pantry-fodmap-friendly</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:08:12.474Z</t>
+  </si>
+  <si>
+    <t>Is Your Pantry FODMAP-Friendly? | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/wellness-tips/is-your-pantry-fodmap-friendly</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/make-a-game-plan-for-ibs-c.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/make-a-game-plan-for-ibs-c</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:07:56.867Z</t>
+  </si>
+  <si>
+    <t>Make a Game Plan for IBS-C | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/wellness-tips/make-a-game-plan-for-ibs-c</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/your-map-to-a-low-fodmap-diet.report.json</t>
+  </si>
+  <si>
+    <t>starting-linzess/wellness-tips/your-map-to-a-low-fodmap-diet</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:07:42.025Z</t>
+  </si>
+  <si>
+    <t>Your Map to a Low FODMAP Diet | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/starting-linzess/wellness-tips/your-map-to-a-low-fodmap-diet</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/could-it-be-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/could-it-be-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:06:21.618Z</t>
+  </si>
+  <si>
+    <t>Could It Be IBS-C or CIC? Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/could-it-be-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/dian-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/dian-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:05:44.977Z</t>
+  </si>
+  <si>
+    <t>Dian Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/dian-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/dr-lucak-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/dr-lucak-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:06:29.632Z</t>
+  </si>
+  <si>
+    <t>Dr. Lucak Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/dr-lucak-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/elaine-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/elaine-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-12T05:10:17.095Z</t>
+  </si>
+  <si>
+    <t>Elaine Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/elaine-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/finding-relief-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/finding-relief-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:06:36.063Z</t>
+  </si>
+  <si>
+    <t>Finding Relief Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/finding-relief-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/getting-on-same-page-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/getting-on-same-page-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:06:06.598Z</t>
+  </si>
+  <si>
+    <t>Getting on the Same Page Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/getting-on-same-page-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/julie-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/julie-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:05:58.566Z</t>
+  </si>
+  <si>
+    <t>Julie Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/julie-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/nan-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/nan-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:05:52.049Z</t>
+  </si>
+  <si>
+    <t>Nan Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/nan-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/seeking-the-right-treatment-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/seeking-the-right-treatment-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:06:44.003Z</t>
+  </si>
+  <si>
+    <t>Seeking the Right Treatment Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/seeking-the-right-treatment-transcripts</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/setting-expectations-transcripts.report.json</t>
+  </si>
+  <si>
+    <t>why-linzess/linzess-patient-experiences/setting-expectations-transcripts</t>
+  </si>
+  <si>
+    <t>2026-06-09T03:06:13.660Z</t>
+  </si>
+  <si>
+    <t>Setting Expectations Transcripts | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/why-linzess/linzess-patient-experiences/setting-expectations-transcripts</t>
   </si>
 </sst>
 </file>
@@ -447,16 +1008,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +1067,968 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
+        <v>74</v>
+      </c>
+      <c r="G13" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>83</v>
+      </c>
+      <c r="G15" t="s">
+        <v>84</v>
+      </c>
+      <c r="H15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" t="s">
+        <v>89</v>
+      </c>
+      <c r="H16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" t="s">
+        <v>94</v>
+      </c>
+      <c r="H17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" t="s">
+        <v>99</v>
+      </c>
+      <c r="H18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>103</v>
+      </c>
+      <c r="G19" t="s">
+        <v>39</v>
+      </c>
+      <c r="H19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
+        <v>107</v>
+      </c>
+      <c r="G20" t="s">
+        <v>39</v>
+      </c>
+      <c r="H20" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" t="s">
+        <v>111</v>
+      </c>
+      <c r="G21" t="s">
+        <v>70</v>
+      </c>
+      <c r="H21" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" t="s">
+        <v>115</v>
+      </c>
+      <c r="G22" t="s">
+        <v>116</v>
+      </c>
+      <c r="H22" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>118</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>119</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" t="s">
+        <v>120</v>
+      </c>
+      <c r="G23" t="s">
+        <v>121</v>
+      </c>
+      <c r="H23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" t="s">
+        <v>124</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" t="s">
+        <v>125</v>
+      </c>
+      <c r="G24" t="s">
+        <v>126</v>
+      </c>
+      <c r="H24" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>128</v>
+      </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>129</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" t="s">
+        <v>130</v>
+      </c>
+      <c r="G25" t="s">
+        <v>131</v>
+      </c>
+      <c r="H25" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" t="s">
+        <v>134</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" t="s">
+        <v>135</v>
+      </c>
+      <c r="G26" t="s">
+        <v>136</v>
+      </c>
+      <c r="H26" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>138</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>139</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" t="s">
+        <v>140</v>
+      </c>
+      <c r="G27" t="s">
+        <v>141</v>
+      </c>
+      <c r="H27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>143</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>144</v>
+      </c>
+      <c r="D28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" t="s">
+        <v>145</v>
+      </c>
+      <c r="G28" t="s">
+        <v>146</v>
+      </c>
+      <c r="H28" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>148</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>149</v>
+      </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" t="s">
+        <v>150</v>
+      </c>
+      <c r="G29" t="s">
+        <v>151</v>
+      </c>
+      <c r="H29" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>153</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>154</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" t="s">
+        <v>155</v>
+      </c>
+      <c r="G30" t="s">
+        <v>156</v>
+      </c>
+      <c r="H30" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>158</v>
+      </c>
+      <c r="B31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" t="s">
+        <v>160</v>
+      </c>
+      <c r="G31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H31" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>163</v>
+      </c>
+      <c r="B32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" t="s">
+        <v>165</v>
+      </c>
+      <c r="G32" t="s">
+        <v>166</v>
+      </c>
+      <c r="H32" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>168</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
+        <v>169</v>
+      </c>
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" t="s">
+        <v>170</v>
+      </c>
+      <c r="G33" t="s">
+        <v>171</v>
+      </c>
+      <c r="H33" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>173</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>174</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" t="s">
+        <v>175</v>
+      </c>
+      <c r="G34" t="s">
+        <v>176</v>
+      </c>
+      <c r="H34" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>178</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>179</v>
+      </c>
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" t="s">
+        <v>180</v>
+      </c>
+      <c r="G35" t="s">
+        <v>181</v>
+      </c>
+      <c r="H35" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>183</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" t="s">
+        <v>184</v>
+      </c>
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>12</v>
+      </c>
+      <c r="F36" t="s">
+        <v>185</v>
+      </c>
+      <c r="G36" t="s">
+        <v>186</v>
+      </c>
+      <c r="H36" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>188</v>
+      </c>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>189</v>
+      </c>
+      <c r="D37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37" t="s">
+        <v>190</v>
+      </c>
+      <c r="G37" t="s">
+        <v>191</v>
+      </c>
+      <c r="H37" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>193</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" t="s">
+        <v>194</v>
+      </c>
+      <c r="D38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" t="s">
+        <v>195</v>
+      </c>
+      <c r="G38" t="s">
+        <v>196</v>
+      </c>
+      <c r="H38" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>198</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" t="s">
+        <v>199</v>
+      </c>
+      <c r="D39" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" t="s">
+        <v>200</v>
+      </c>
+      <c r="G39" t="s">
+        <v>201</v>
+      </c>
+      <c r="H39" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>